<commit_message>
docs(sessions): business plan v3 for CasaZen as a product
Drop partner-specific content (offer, framework contract, pilot and
migration of a named agency) and describe the first Founding Partner
generically. Keep the numbers: the first Founding Partner is modelled as
a 250-unit agency with a pilot and a progressive migration.

Claude-Session: https://claude.ai/code/session_011LxaCT2ysBgYUs8soVaYPm
</commit_message>
<xml_diff>
--- a/Sessions/business-plan-2026-10/modello/modello-economico.xlsx
+++ b/Sessions/business-plan-2026-10/modello/modello-economico.xlsx
@@ -105,7 +105,7 @@
     <t xml:space="preserve">Scenari</t>
   </si>
   <si>
-    <t xml:space="preserve">A. Solo Quokka</t>
+    <t xml:space="preserve">A. Solo il primo Founding Partner</t>
   </si>
   <si>
     <t xml:space="preserve">B. Ritardo</t>
@@ -117,10 +117,10 @@
     <t xml:space="preserve">Attivo</t>
   </si>
   <si>
-    <t xml:space="preserve">Mese di avvio del pilota Quokka (99999 = mai)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unità Quokka a regime</t>
+    <t xml:space="preserve">Primo Founding Partner: mese di avvio del pilota (99999 = mai)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primo Founding Partner: unità a regime</t>
   </si>
   <si>
     <t xml:space="preserve">Unità del pilota</t>
@@ -138,7 +138,7 @@
     <t xml:space="preserve">Primo mese altri Founding Partner</t>
   </si>
   <si>
-    <t xml:space="preserve">Posti Founding Partner oltre Quokka</t>
+    <t xml:space="preserve">Posti Founding Partner oltre il primo</t>
   </si>
   <si>
     <t xml:space="preserve">Nuovi Founding Partner al mese</t>
@@ -288,13 +288,13 @@
     <t xml:space="preserve">Indice mese</t>
   </si>
   <si>
-    <t xml:space="preserve">Pilota Quokka avviato (1/0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quokka a regime (1/0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unità Quokka</t>
+    <t xml:space="preserve">Pilota del primo FP avviato (1/0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primo FP a regime (1/0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unità del primo Founding Partner</t>
   </si>
   <si>
     <t xml:space="preserve">Altri Founding Partner (agenzie)</t>

</xml_diff>